<commit_message>
added lsm6dsl to pcb and ordered v3
</commit_message>
<xml_diff>
--- a/pcb/stm32f765-breakout-board/breakout_board_bom.xlsx
+++ b/pcb/stm32f765-breakout-board/breakout_board_bom.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="82">
   <si>
     <t xml:space="preserve">Robu SKU</t>
   </si>
@@ -71,6 +71,9 @@
   </si>
   <si>
     <t xml:space="preserve">10n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R139421</t>
   </si>
   <si>
     <t xml:space="preserve">C11,C12</t>
@@ -277,6 +280,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -298,6 +302,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -342,24 +347,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -486,687 +495,779 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="4.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="59.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.31"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="2" min="2" style="1" width="28.98"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="3" min="3" style="1" width="4.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15.34"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="5" min="5" style="1" width="59.17"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>595331</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="G2" s="0" t="n">
+      <c r="E2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="G2" s="1" t="n">
         <v>1.8</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="H2" s="4" t="n">
         <f aca="false">G2*F2</f>
         <v>18</v>
       </c>
+      <c r="I2" s="0" t="n">
+        <f aca="false">H2</f>
+        <v>18</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>595344</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="0" t="n">
+      <c r="E3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="G3" s="0" t="n">
+      <c r="G3" s="1" t="n">
         <v>0.7</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="H3" s="4" t="n">
         <f aca="false">G3*F3</f>
         <v>35</v>
       </c>
+      <c r="I3" s="0" t="n">
+        <f aca="false">H3+I2</f>
+        <v>53</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>1544904</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="0" t="s">
+      <c r="C4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="G4" s="0" t="n">
+      <c r="E4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="G4" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="H4" s="4" t="n">
         <f aca="false">G4*F4</f>
         <v>130</v>
       </c>
+      <c r="I4" s="0" t="n">
+        <f aca="false">H4+I3</f>
+        <v>183</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>595338</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="0" t="s">
+      <c r="C5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="G5" s="0" t="n">
+      <c r="E5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="G5" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="H5" s="4" t="n">
         <f aca="false">G5*F5</f>
         <v>50</v>
       </c>
+      <c r="I5" s="0" t="n">
+        <f aca="false">H5+I4</f>
+        <v>233</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="n">
-        <v>1089873</v>
-      </c>
-      <c r="B6" s="0" t="s">
+      <c r="A6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="0" t="n">
+      <c r="B6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="0" t="n">
+      <c r="D6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="G6" s="0" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="H6" s="3" t="n">
+      <c r="G6" s="1" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="H6" s="4" t="n">
         <f aca="false">G6*F6</f>
-        <v>34.8</v>
+        <v>26.8</v>
+      </c>
+      <c r="I6" s="0" t="n">
+        <f aca="false">H6+I5</f>
+        <v>259.8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="0" t="s">
+      <c r="A7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="0" t="n">
+      <c r="B7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="0" t="n">
+      <c r="D7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="G7" s="0" t="n">
+      <c r="G7" s="1" t="n">
         <v>1.86</v>
       </c>
-      <c r="H7" s="3" t="n">
+      <c r="H7" s="4" t="n">
         <f aca="false">G7*F7</f>
         <v>37.2</v>
       </c>
+      <c r="I7" s="0" t="n">
+        <f aca="false">H7+I6</f>
+        <v>297</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="3" t="n">
         <v>827887</v>
       </c>
-      <c r="B8" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="C8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F8" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="G8" s="0" t="n">
+      <c r="E8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="G8" s="1" t="n">
         <v>0.79</v>
       </c>
-      <c r="H8" s="3" t="n">
+      <c r="H8" s="4" t="n">
         <f aca="false">G8*F8</f>
-        <v>7.9</v>
+        <v>15.8</v>
+      </c>
+      <c r="I8" s="0" t="n">
+        <f aca="false">H8+I7</f>
+        <v>312.8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="0" t="s">
+      <c r="A9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="C9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F9" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="G9" s="0" t="n">
+      <c r="E9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="H9" s="3" t="n">
+      <c r="H9" s="4" t="n">
         <f aca="false">G9*F9</f>
         <v>30</v>
       </c>
+      <c r="I9" s="0" t="n">
+        <f aca="false">H9+I8</f>
+        <v>342.8</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="B10" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="E10" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="F10" s="0" t="n">
+      <c r="H10" s="4" t="n">
+        <f aca="false">G10*F10</f>
+        <v>290</v>
+      </c>
+      <c r="I10" s="0" t="n">
+        <f aca="false">H10+I9</f>
+        <v>632.8</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="n">
+        <v>1114172</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="G10" s="0" t="n">
+      <c r="G11" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <f aca="false">G11*F11</f>
+        <v>25</v>
+      </c>
+      <c r="I11" s="0" t="n">
+        <f aca="false">H11+I10</f>
+        <v>657.8</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="n">
+        <v>1114172</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H10" s="3" t="n">
-        <f aca="false">G10*F10</f>
-        <v>190</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="n">
+      <c r="E12" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <f aca="false">G12*F12</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="0" t="n">
+        <f aca="false">H12+I11</f>
+        <v>657.8</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="n">
         <v>1114172</v>
       </c>
-      <c r="B11" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="F11" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="0" t="n">
+      <c r="B13" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="H11" s="3" t="n">
-        <f aca="false">G11*F11</f>
+      <c r="H13" s="4" t="n">
+        <f aca="false">G13*F13</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="0" t="n">
+        <f aca="false">H13+I12</f>
+        <v>657.8</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="n">
+        <v>1114172</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="1" t="n">
         <v>5</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="n">
+      <c r="H14" s="4" t="n">
+        <f aca="false">G14*F14</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="0" t="n">
+        <f aca="false">H14+I13</f>
+        <v>657.8</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="n">
         <v>1114172</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B15" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <f aca="false">G15*F15</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="0" t="n">
+        <f aca="false">H15+I14</f>
+        <v>657.8</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="n">
+        <v>1114172</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="E12" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="F12" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="0" t="n">
+      <c r="F16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="H12" s="3" t="n">
-        <f aca="false">G12*F12</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="n">
-        <v>1114172</v>
-      </c>
-      <c r="B13" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="E13" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="F13" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="H13" s="3" t="n">
-        <f aca="false">G13*F13</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="n">
-        <v>1114172</v>
-      </c>
-      <c r="B14" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="E14" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="F14" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="H14" s="3" t="n">
-        <f aca="false">G14*F14</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="n">
-        <v>1114172</v>
-      </c>
-      <c r="B15" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="C15" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="E15" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="F15" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="H15" s="3" t="n">
-        <f aca="false">G15*F15</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="n">
-        <v>1114172</v>
-      </c>
-      <c r="B16" s="0" t="s">
-        <v>47</v>
-      </c>
-      <c r="C16" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="E16" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="F16" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="H16" s="3" t="n">
+      <c r="H16" s="4" t="n">
         <f aca="false">G16*F16</f>
         <v>0</v>
       </c>
+      <c r="I16" s="0" t="n">
+        <f aca="false">H16+I15</f>
+        <v>657.8</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B17" s="0" t="s">
+      <c r="A17" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C17" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="0" t="s">
+      <c r="C17" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F17" s="0" t="n">
+      <c r="E17" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F17" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G17" s="0" t="n">
+      <c r="G17" s="1" t="n">
         <v>0.16</v>
       </c>
-      <c r="H17" s="3" t="n">
+      <c r="H17" s="4" t="n">
         <f aca="false">G17*F17</f>
         <v>16</v>
       </c>
+      <c r="I17" s="0" t="n">
+        <f aca="false">H17+I16</f>
+        <v>673.8</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="0" t="s">
-        <v>54</v>
-      </c>
-      <c r="C18" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="D18" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="E18" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="F18" s="0" t="n">
+      <c r="F18" s="1" t="n">
         <v>100</v>
       </c>
-      <c r="G18" s="0" t="n">
+      <c r="G18" s="1" t="n">
         <v>0.28</v>
       </c>
-      <c r="H18" s="3" t="n">
+      <c r="H18" s="4" t="n">
         <f aca="false">G18*F18</f>
         <v>28</v>
       </c>
+      <c r="I18" s="0" t="n">
+        <f aca="false">H18+I17</f>
+        <v>701.8</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B19" s="0" t="s">
+      <c r="A19" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C19" s="0" t="n">
+      <c r="B19" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C19" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D19" s="0" t="s">
-        <v>58</v>
-      </c>
-      <c r="E19" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="F19" s="0" t="n">
+      <c r="D19" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="G19" s="0" t="n">
+      <c r="G19" s="1" t="n">
         <v>0.68</v>
       </c>
-      <c r="H19" s="3" t="n">
+      <c r="H19" s="4" t="n">
         <f aca="false">G19*F19</f>
         <v>34</v>
       </c>
+      <c r="I19" s="0" t="n">
+        <f aca="false">H19+I18</f>
+        <v>735.8</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="3" t="n">
         <v>1883759</v>
       </c>
-      <c r="B20" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="C20" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E20" s="0" t="s">
+      <c r="C20" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F20" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="G20" s="0" t="n">
+      <c r="E20" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G20" s="1" t="n">
         <v>1.55</v>
       </c>
-      <c r="H20" s="3" t="n">
+      <c r="H20" s="4" t="n">
         <f aca="false">G20*F20</f>
         <v>15.5</v>
       </c>
+      <c r="I20" s="0" t="n">
+        <f aca="false">H20+I19</f>
+        <v>751.3</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B21" s="0" t="s">
+      <c r="A21" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C21" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="E21" s="0" t="s">
+      <c r="C21" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="F21" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="0" t="n">
+      <c r="E21" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F21" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="1" t="n">
         <v>794</v>
       </c>
-      <c r="H21" s="3" t="n">
+      <c r="H21" s="4" t="n">
         <f aca="false">G21*F21</f>
-        <v>794</v>
+        <v>1588</v>
+      </c>
+      <c r="I21" s="0" t="n">
+        <f aca="false">H21+I20</f>
+        <v>2339.3</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B22" s="0" t="s">
+      <c r="A22" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C22" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E22" s="0" t="s">
+      <c r="C22" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F22" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="G22" s="0" t="n">
+      <c r="E22" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F22" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="G22" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="H22" s="3" t="n">
+      <c r="H22" s="4" t="n">
         <f aca="false">G22*F22</f>
         <v>70</v>
       </c>
+      <c r="I22" s="0" t="n">
+        <f aca="false">H22+I21</f>
+        <v>2409.3</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="B23" s="0" t="s">
+      <c r="A23" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C23" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E23" s="0" t="s">
+      <c r="C23" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F23" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="G23" s="0" t="n">
+      <c r="E23" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F23" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="G23" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="H23" s="3" t="n">
+      <c r="H23" s="4" t="n">
         <f aca="false">G23*F23</f>
         <v>60</v>
       </c>
+      <c r="I23" s="0" t="n">
+        <f aca="false">H23+I22</f>
+        <v>2469.3</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B24" s="0" t="s">
+      <c r="A24" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E24" s="0" t="s">
+      <c r="C24" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="F24" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="G24" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="H24" s="3" t="n">
+      <c r="E24" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F24" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="G24" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="H24" s="4" t="n">
         <f aca="false">G24*F24</f>
         <v>100</v>
       </c>
+      <c r="I24" s="0" t="n">
+        <f aca="false">H24+I23</f>
+        <v>2569.3</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G25" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="H25" s="1" t="n">
+      <c r="G25" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H25" s="2" t="n">
         <f aca="false">SUM(H2:H24)</f>
-        <v>1675.4</v>
+        <v>2569.3</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G26" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="H26" s="1" t="n">
+      <c r="G26" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="H26" s="2" t="n">
         <v>981</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G27" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="H27" s="1" t="n">
+      <c r="G27" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="H27" s="2" t="n">
         <f aca="false">SUM(H25:H26)</f>
-        <v>2656.4</v>
+        <v>3550.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>